<commit_message>
Report missing database entries in texture classification hook; add texture utility data
- _Insert_derived_classifications runs classifiers first and prints a
  compulsory, once-per-run ERROR (any verbosity, import continues) when
  texture is derivable but no class indicator is registered, when a
  provision_indicator lacks an analysis_method (previously a crash), or
  when a derived class has no nominal_classification row.
- New _Diagnose_classification_indicators walks quantity 'class' ->
  indicator -> provision_indicator and lists what is missing.
- Utility data: quantity/unit 'class', four soil texture indicators,
  nominal_classes.xlsx, texture provision_indicator rows for agrolab,
  veltia and ibec; nominal_classes.json added to the insert pilot list.

import_data.py and pg_ai4sh.py kept identical with xspatula_lucas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ai4sh/import_data/utility/observation/excel/indicator.xlsx
+++ b/ai4sh/import_data/utility/observation/excel/indicator.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="234">
   <si>
     <t xml:space="preserve">quantity_id__quantity_name</t>
   </si>
@@ -665,6 +665,63 @@
   </si>
   <si>
     <t xml:space="preserve">Bacteria relative microbial content</t>
+  </si>
+  <si>
+    <t xml:space="preserve">class</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Classification with nominative value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">soil texture class iuss</t>
+  </si>
+  <si>
+    <t xml:space="preserve">soil texture iuss</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Soil texture class IUSS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IUSS soil texture classification</t>
+  </si>
+  <si>
+    <t xml:space="preserve">soil texture class usda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">soil texture usda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Soil texture class USDA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USDA soil texture classification</t>
+  </si>
+  <si>
+    <t xml:space="preserve">soil texture class usda major group</t>
+  </si>
+  <si>
+    <t xml:space="preserve">soil texture usda major group</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Soil texture usda major group</t>
+  </si>
+  <si>
+    <t xml:space="preserve">soil texture class iuss major group</t>
+  </si>
+  <si>
+    <t xml:space="preserve">soil texture iuss major group</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Soil texture iuss major group</t>
+  </si>
+  <si>
+    <t xml:space="preserve">compilation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compilation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compilation of 2 or more source datasets to a single dataset</t>
   </si>
 </sst>
 </file>
@@ -957,7 +1014,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E89"/>
+  <dimension ref="A1:E95"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="43.36"/>
@@ -2238,6 +2295,102 @@
         <v>214</v>
       </c>
     </row>
+    <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="C90" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="D90" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="E90" s="1" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="C91" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="D91" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="E91" s="1" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="C92" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="D92" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="E92" s="1" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="B93" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="C93" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="D93" s="2" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="B94" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="C94" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="D94" s="2" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="B95" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="C95" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="D95" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="E95" s="1" t="s">
+        <v>233</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>

</xml_diff>